<commit_message>
scan: seg7 2026-08-11 16:11 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-08-11.xlsx
+++ b/output/full_scan/batch_seq8_2026-08-11.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O126"/>
+  <dimension ref="A1:O128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3230,21 +3230,21 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6994</v>
+        <v>7610</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>富威電力</t>
+          <t>聯友金屬-創</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>323.8803356481768</v>
+        <v>324.4279036238797</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>36.3</v>
+        <v>1870</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>30.99490220112421</v>
+        <v>52.63649558397829</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>37.56357397224496</v>
+        <v>26.48273230206593</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>1.590546610593683</v>
+        <v>0.2785460516226864</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.317302916605124</v>
+        <v>48.33171541543968</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6918</v>
+        <v>6994</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>愛派司</t>
+          <t>富威電力</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>322.5672136981403</v>
+        <v>323.8803356481768</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>73.8</v>
+        <v>36.3</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>56.65806188896151</v>
+        <v>30.99490220112421</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>16.00214407632894</v>
+        <v>37.56357397224496</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>1.284953335936545</v>
+        <v>1.590546610593683</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.2602308793995962</v>
+        <v>0.317302916605124</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, cci_momentum</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6919</v>
+        <v>6918</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>康霈*</t>
+          <t>愛派司</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>320.2093858909667</v>
+        <v>322.5672136981403</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>108</v>
+        <v>73.8</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>53.92750906854776</v>
+        <v>56.65806188896151</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>18.20476266159357</v>
+        <v>16.00214407632894</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.6087717031030908</v>
+        <v>1.284953335936545</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.368715559603689</v>
+        <v>0.2602308793995962</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6931</v>
+        <v>6919</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>青松健康</t>
+          <t>康霈*</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>317.2542818767268</v>
+        <v>320.2093858909667</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>39.5</v>
+        <v>108</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>55.37704646686871</v>
+        <v>53.92750906854776</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>19.7833755470187</v>
+        <v>18.20476266159357</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1.362574799460546</v>
+        <v>0.6087717031030908</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.1853969327605436</v>
+        <v>0.368715559603689</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6910</v>
+        <v>6931</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>德鴻</t>
+          <t>青松健康</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>316.3166301572181</v>
+        <v>317.2542818767268</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>25.1</v>
+        <v>39.5</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>46.66960512757235</v>
+        <v>55.37704646686871</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>24.21464755664187</v>
+        <v>19.7833755470187</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.4752970606629143</v>
+        <v>1.362574799460546</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.1723280828385345</v>
+        <v>0.1853969327605436</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>7738</v>
+        <v>6910</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>東聯互動</t>
+          <t>德鴻</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>309.0248703271594</v>
+        <v>316.3166301572181</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>169</v>
+        <v>25.1</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>53.75912477615551</v>
+        <v>46.66960512757235</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>30.69405483610011</v>
+        <v>24.21464755664187</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.5453129940199155</v>
+        <v>0.4752970606629143</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.4127997871577152</v>
+        <v>0.1723280828385345</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>8040</v>
+        <v>8021</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>九暘</t>
+          <t>尖點</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>308.8686672090263</v>
+        <v>310.1626457524277</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>74.7</v>
+        <v>439</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>45.3461432305179</v>
+        <v>52.66185451715562</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>24.61598696895319</v>
+        <v>19.33156420632769</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.4259122490862397</v>
+        <v>0.260131384231533</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>1.53869259162726</v>
+        <v>11.60275452703239</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6967</v>
+        <v>7738</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>東聯互動</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>306.6671869416742</v>
+        <v>309.0248703271594</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>68.7</v>
+        <v>169</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>44.10272818206129</v>
+        <v>53.75912477615551</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>16.64185833357534</v>
+        <v>30.69405483610011</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.3002015540373611</v>
+        <v>0.5453129940199155</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.2527641638728034</v>
+        <v>0.4127997871577152</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>8038</v>
+        <v>8040</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>長園科</t>
+          <t>九暘</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>306.3647806188447</v>
+        <v>308.8686672090263</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>32.45</v>
+        <v>74.7</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>37.45047521381427</v>
+        <v>45.3461432305179</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>20.6456835337207</v>
+        <v>24.61598696895319</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.7264050234239444</v>
+        <v>0.4259122490862397</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>2</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.0499294309119981</v>
+        <v>1.53869259162726</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>7827</v>
+        <v>6967</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>漢康-KY創</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>304.9215653678002</v>
+        <v>306.6671869416742</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>161</v>
+        <v>68.7</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>56.41884547384961</v>
+        <v>44.10272818206129</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>14.42040685956114</v>
+        <v>16.64185833357534</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.509189667044939</v>
+        <v>0.3002015540373611</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>1.783930461999255</v>
+        <v>-0.2527641638728034</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>8034</v>
+        <v>8038</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>榮群</t>
+          <t>長園科</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>303.9153426762072</v>
+        <v>306.3647806188447</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>18.9</v>
+        <v>32.45</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>38.09941254792758</v>
+        <v>37.45047521381427</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>36.0499560774052</v>
+        <v>20.6456835337207</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.7370511468511693</v>
+        <v>0.7264050234239444</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.1278623497031097</v>
+        <v>0.0499294309119981</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>7730</v>
+        <v>7827</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>暉盛-創</t>
+          <t>漢康-KY創</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>302.5179802339178</v>
+        <v>304.9215653678002</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>49.00335099683544</v>
+        <v>56.41884547384961</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>25.68287863657897</v>
+        <v>14.42040685956114</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>1.013271617345562</v>
+        <v>0.509189667044939</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>1.278075785083636</v>
+        <v>1.783930461999255</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>7721</v>
+        <v>8034</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>微程式</t>
+          <t>榮群</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>290.9538476004316</v>
+        <v>303.9153426762072</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>63.2</v>
+        <v>18.9</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,16 +3891,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>47.81269872857953</v>
+        <v>38.09941254792758</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>24.71147806414012</v>
+        <v>36.0499560774052</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.4233919008741237</v>
+        <v>0.7370511468511693</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.8164423856988652</v>
+        <v>0.1278623497031097</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6865</v>
+        <v>7730</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>偉康科技</t>
+          <t>暉盛-創</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>288.9064812071622</v>
+        <v>302.5179802339178</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>25.25</v>
+        <v>163</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>51.37607364624409</v>
+        <v>49.00335099683544</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>8.081846029526627</v>
+        <v>25.68287863657897</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.5021984126236901</v>
+        <v>1.013271617345562</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.7859925030937126</v>
+        <v>1.278075785083636</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>7556</v>
+        <v>7721</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>意德士</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>287.1002318780993</v>
+        <v>290.9538476004316</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>223</v>
+        <v>63.2</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>44.06656300526173</v>
+        <v>47.81269872857953</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>33.25791802222026</v>
+        <v>24.71147806414012</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.520540478160626</v>
+        <v>0.4233919008741237</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>3.30067555979868</v>
+        <v>0.8164423856988652</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6840</v>
+        <v>6865</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>東研信超</t>
+          <t>偉康科技</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>286.4616688110532</v>
+        <v>288.9064812071622</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>68</v>
+        <v>25.25</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>61.90067115938755</v>
+        <v>51.37607364624409</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>16.5986358827138</v>
+        <v>8.081846029526627</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.8633751384931831</v>
+        <v>0.5021984126236901</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>1.00381250404702</v>
+        <v>0.7859925030937126</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6901</v>
+        <v>7556</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>鑽石投資</t>
+          <t>意德士</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>282.409282418675</v>
+        <v>287.1002318780993</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>16.85</v>
+        <v>223</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>47.19136307998259</v>
+        <v>44.06656300526173</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>19.6752956335989</v>
+        <v>33.25791802222026</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>1.909899586141167</v>
+        <v>0.520540478160626</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.0755863099839509</v>
+        <v>3.30067555979868</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6996</v>
+        <v>6840</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>力領科技</t>
+          <t>東研信超</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>278.0265149014633</v>
+        <v>286.4616688110532</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>176.5</v>
+        <v>68</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>46.32390375607011</v>
+        <v>61.90067115938755</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>18.43884116102049</v>
+        <v>16.5986358827138</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.4718833860870829</v>
+        <v>0.8633751384931831</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>1.330692858469333</v>
+        <v>1.00381250404702</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6877</v>
+        <v>6901</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>鏵友益</t>
+          <t>鑽石投資</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>274.9952449562192</v>
+        <v>282.409282418675</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>127.5</v>
+        <v>16.85</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>52.24148098522304</v>
+        <v>47.19136307998259</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>17.65562995298108</v>
+        <v>19.6752956335989</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.4207206625835656</v>
+        <v>1.909899586141167</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>1.714243405380859</v>
+        <v>-0.0755863099839509</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6936</v>
+        <v>6996</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>永鴻生技</t>
+          <t>力領科技</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>271.0169993515908</v>
+        <v>278.0265149014633</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>32.05</v>
+        <v>176.5</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>48.34777283661477</v>
+        <v>46.32390375607011</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>13.08771940582141</v>
+        <v>18.43884116102049</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.548108034928586</v>
+        <v>0.4718833860870829</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0764888007585085</v>
+        <v>1.330692858469333</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>7732</v>
+        <v>6877</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>金興精密</t>
+          <t>鏵友益</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>261.440040109625</v>
+        <v>274.9952449562192</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>34.7</v>
+        <v>127.5</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>49.68908740826368</v>
+        <v>52.24148098522304</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>3.710488400137273</v>
+        <v>17.65562995298108</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>2.165453375878123</v>
+        <v>0.4207206625835656</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.1558968677075366</v>
+        <v>1.714243405380859</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>7768</v>
+        <v>6936</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>頌勝科技</t>
+          <t>永鴻生技</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>261.268695404051</v>
+        <v>271.0169993515908</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>256.5</v>
+        <v>32.05</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>34.16142446675504</v>
+        <v>48.34777283661477</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>45.46295401723033</v>
+        <v>13.08771940582141</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.5968418158309151</v>
+        <v>0.548108034928586</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>2.292043060626078</v>
+        <v>0.0764888007585085</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6951</v>
+        <v>7732</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>青新-創</t>
+          <t>金興精密</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>256.0458413928027</v>
+        <v>261.440040109625</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>71.40000000000001</v>
+        <v>34.7</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>38.0619752064248</v>
+        <v>49.68908740826368</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>37.35877948247683</v>
+        <v>3.710488400137273</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.2097988721191772</v>
+        <v>2.165453375878123</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.258872344223916</v>
+        <v>-0.1558968677075366</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>7855</v>
+        <v>7768</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>和運租車</t>
+          <t>頌勝科技</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>256</v>
+        <v>261.268695404051</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>43.75</v>
+        <v>256.5</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>17.1498013016375</v>
+        <v>34.16142446675504</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>20.6428621797185</v>
+        <v>45.46295401723033</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>18.62803994913243</v>
+        <v>0.5968418158309151</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-4.482763329033666</v>
+        <v>2.292043060626078</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6965</v>
+        <v>6951</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>青新-創</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>254.3814201463255</v>
+        <v>256.0458413928027</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>75.90000000000001</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>40.55012652608201</v>
+        <v>38.0619752064248</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>32.05390748338364</v>
+        <v>37.35877948247683</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>1.361791559624175</v>
+        <v>0.2097988721191772</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.1258160348789537</v>
+        <v>0.258872344223916</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4555,21 +4555,21 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6906</v>
+        <v>7855</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>現觀科</t>
+          <t>和運租車</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>253.3727773791067</v>
+        <v>256</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>72.5</v>
+        <v>43.75</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>45.02221552301081</v>
+        <v>17.1498013016375</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>28.21163581573396</v>
+        <v>20.6428621797185</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>1.061110119633245</v>
+        <v>18.62803994913243</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.8937304799819996</v>
+        <v>-4.482763329033666</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, kd_golden_cross</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6947</v>
+        <v>6965</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>台鎔科技</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>246.9770270171257</v>
+        <v>254.3814201463255</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>76</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>44.39314939210099</v>
+        <v>40.55012652608201</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>19.11705830915324</v>
+        <v>32.05390748338364</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.3910575165099926</v>
+        <v>1.361791559624175</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.7736619760815149</v>
+        <v>-0.1258160348789537</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>8028</v>
+        <v>6906</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>昇陽半導體</t>
+          <t>現觀科</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>246.921233633889</v>
+        <v>253.3727773791067</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>261</v>
+        <v>72.5</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>43.82629621728131</v>
+        <v>45.02221552301081</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>17.57046314374402</v>
+        <v>28.21163581573396</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.519461077170339</v>
+        <v>1.061110119633245</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-1.303939384191921</v>
+        <v>0.8937304799819996</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>7803</v>
+        <v>6947</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>雲象科技-創</t>
+          <t>台鎔科技</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>246.7822462983393</v>
+        <v>246.9770270171257</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>19.75</v>
+        <v>76</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>39.11479271648616</v>
+        <v>44.39314939210099</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>21.25737262354921</v>
+        <v>19.11705830915324</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.1365588774461856</v>
+        <v>0.3910575165099926</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0591232067974026</v>
+        <v>0.7736619760815149</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>7780</v>
+        <v>8028</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>大研生醫*</t>
+          <t>昇陽半導體</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>246.1104869916361</v>
+        <v>246.921233633889</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>16.8</v>
+        <v>261</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>38.15183731014595</v>
+        <v>43.82629621728131</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>34.16086084716387</v>
+        <v>17.57046314374402</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.5415617086820069</v>
+        <v>0.519461077170339</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.026517068273454</v>
+        <v>-1.303939384191921</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6890</v>
+        <v>7803</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>來億-KY</t>
+          <t>雲象科技-創</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>241.3621174638651</v>
+        <v>246.7822462983393</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>174.5</v>
+        <v>19.75</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>45.23382973208128</v>
+        <v>39.11479271648616</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>12.65930992128667</v>
+        <v>21.25737262354921</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.3314200698822124</v>
+        <v>0.1365588774461856</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>1.875751219518275</v>
+        <v>0.0591232067974026</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>7722</v>
+        <v>7780</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>LINEPAY</t>
+          <t>大研生醫*</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>239.3220254637132</v>
+        <v>246.1104869916361</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>291.5</v>
+        <v>16.8</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>49.73832241201093</v>
+        <v>38.15183731014595</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>21.59265261953322</v>
+        <v>34.16086084716387</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.367492021236368</v>
+        <v>0.5415617086820069</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>1.834703384881334</v>
+        <v>0.026517068273454</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>7799</v>
+        <v>6890</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>禾榮科</t>
+          <t>來億-KY</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>239.0998250197794</v>
+        <v>241.3621174638651</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>359</v>
+        <v>174.5</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>43.39148713474725</v>
+        <v>45.23382973208128</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>20.59127055498088</v>
+        <v>12.65930992128667</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.3428285191706263</v>
+        <v>0.3314200698822124</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-2.518695951257056</v>
+        <v>1.875751219518275</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6873</v>
+        <v>7722</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>LINEPAY</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>236.1849586711393</v>
+        <v>239.3220254637132</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>74.8</v>
+        <v>291.5</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>35.70210164367053</v>
+        <v>49.73832241201093</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>17.43112291946078</v>
+        <v>21.59265261953322</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>2.621261352234333</v>
+        <v>0.367492021236368</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.4726511434196982</v>
+        <v>1.834703384881334</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6869</v>
+        <v>7799</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>雲豹能源</t>
+          <t>禾榮科</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>232.5715648458117</v>
+        <v>239.0998250197794</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>67.3</v>
+        <v>359</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>44.13250447780238</v>
+        <v>43.39148713474725</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>18.43993606883123</v>
+        <v>20.59127055498088</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.6275990503118812</v>
+        <v>0.3428285191706263</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.6031818358028298</v>
+        <v>-2.518695951257056</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>7792</v>
+        <v>6873</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>安葆</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>230.948565364882</v>
+        <v>236.1849586711393</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>211.5</v>
+        <v>74.8</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>46.39302379220982</v>
+        <v>35.70210164367053</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>29.44439325243127</v>
+        <v>17.43112291946078</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.7107049018697245</v>
+        <v>2.621261352234333</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>3.627058829731008</v>
+        <v>-0.4726511434196982</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>7749</v>
+        <v>6869</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>雲豹能源</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>229.7377718036324</v>
+        <v>232.5715648458117</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>359.5</v>
+        <v>67.3</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>46.33436255707659</v>
+        <v>44.13250447780238</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>31.16310653768807</v>
+        <v>18.43993606883123</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.5173385046834837</v>
+        <v>0.6275990503118812</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>6.317538948270531</v>
+        <v>0.6031818358028298</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6859</v>
+        <v>7792</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>伯特光</t>
+          <t>安葆</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>229.1274857117959</v>
+        <v>230.948565364882</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>99.2</v>
+        <v>211.5</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>35.66412797047811</v>
+        <v>46.39302379220982</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>27.68049437065917</v>
+        <v>29.44439325243127</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.4480585922774516</v>
+        <v>0.7107049018697245</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.9394589651827534</v>
+        <v>3.627058829731008</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6934</v>
+        <v>7749</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>心誠鎂</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>222.6470469207084</v>
+        <v>229.7377718036324</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>72.5</v>
+        <v>359.5</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>44.4856215316977</v>
+        <v>46.33436255707659</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>17.36267837071677</v>
+        <v>31.16310653768807</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>1.198601973684211</v>
+        <v>0.5173385046834837</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.7611766531987858</v>
+        <v>6.317538948270531</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>8024</v>
+        <v>6859</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>佑華</t>
+          <t>伯特光</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>220.1334953149262</v>
+        <v>229.1274857117959</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>13.8</v>
+        <v>99.2</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>41.71054769576779</v>
+        <v>35.66412797047811</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>17.34720052770448</v>
+        <v>27.68049437065917</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.753759353792649</v>
+        <v>0.4480585922774516</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.1463191595500006</v>
+        <v>0.9394589651827534</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>7842</v>
+        <v>6934</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>心誠鎂</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>212.7984579954426</v>
+        <v>222.6470469207084</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>94</v>
+        <v>72.5</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>54.31749663823657</v>
+        <v>44.4856215316977</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>10.66722445620016</v>
+        <v>17.36267837071677</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>3.21661227373806</v>
+        <v>1.198601973684211</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>1.907900389183593</v>
+        <v>-0.7611766531987858</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6887</v>
+        <v>8024</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>寶綠特-KY</t>
+          <t>佑華</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>211.68617814312</v>
+        <v>220.1334953149262</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>36.45</v>
+        <v>13.8</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>49.31695248432469</v>
+        <v>41.71054769576779</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>17.04578355064413</v>
+        <v>17.34720052770448</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.1825626148277355</v>
+        <v>0.753759353792649</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.1819288498890896</v>
+        <v>-0.1463191595500006</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6894</v>
+        <v>7842</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>衛司特</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>208.873830439202</v>
+        <v>212.7984579954426</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>345</v>
+        <v>94</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>52.3219923856823</v>
+        <v>54.31749663823657</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>15.45647148628926</v>
+        <v>10.66722445620016</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.8203025307091175</v>
+        <v>3.21661227373806</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>4.056701308693365</v>
+        <v>1.907900389183593</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6916</v>
+        <v>6887</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>寶綠特-KY</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>204.5744204188318</v>
+        <v>211.68617814312</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>18.7</v>
+        <v>36.45</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>47.58853670104529</v>
+        <v>49.31695248432469</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>13.81213421387869</v>
+        <v>17.04578355064413</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.200521903827872</v>
+        <v>0.1825626148277355</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0527311534019029</v>
+        <v>-0.1819288498890896</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6953</v>
+        <v>6894</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>衛司特</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>204.1981402739606</v>
+        <v>208.873830439202</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>220.5</v>
+        <v>345</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>51.07536084264394</v>
+        <v>52.3219923856823</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>9.407512687987516</v>
+        <v>15.45647148628926</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.1880072290599755</v>
+        <v>0.8203025307091175</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>2.04210416579964</v>
+        <v>4.056701308693365</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6988</v>
+        <v>6916</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>威力暘-創</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>203.5494061530428</v>
+        <v>204.5744204188318</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>12.7</v>
+        <v>18.7</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>50.98520902686534</v>
+        <v>47.58853670104529</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>10.68239455268137</v>
+        <v>13.81213421387869</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.9285713101312104</v>
+        <v>0.200521903827872</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.2437915569015741</v>
+        <v>0.0527311534019029</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6899</v>
+        <v>6953</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>203.317649325788</v>
+        <v>204.1981402739606</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>51</v>
+        <v>220.5</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>40.48779896859401</v>
+        <v>51.07536084264394</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>22.59476417999487</v>
+        <v>9.407512687987516</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.5579291095827936</v>
+        <v>0.1880072290599755</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.3811609168553613</v>
+        <v>2.04210416579964</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>7791</v>
+        <v>6988</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>威力暘-創</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>195.5050053759604</v>
+        <v>203.5494061530428</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>59.5</v>
+        <v>12.7</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>31.9038991525452</v>
+        <v>50.98520902686534</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>25.76078683036973</v>
+        <v>10.68239455268137</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.424318686171579</v>
+        <v>0.9285713101312104</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.08340806992414471</v>
+        <v>0.2437915569015741</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>7818</v>
+        <v>6899</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>191.0739285069669</v>
+        <v>203.317649325788</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>35.60140952595299</v>
+        <v>40.48779896859401</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>33.29886568889377</v>
+        <v>22.59476417999487</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.5424617741357679</v>
+        <v>0.5579291095827936</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.334856587748253</v>
+        <v>0.3811609168553613</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5827,21 +5827,21 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6854</v>
+        <v>7791</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>190.2200182423165</v>
+        <v>195.5050053759604</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>93.7</v>
+        <v>59.5</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>36.717587193692</v>
+        <v>31.9038991525452</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>38.9643703424982</v>
+        <v>25.76078683036973</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.2039096226856182</v>
+        <v>0.424318686171579</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>1.47187137430882</v>
+        <v>-0.08340806992414471</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5880,21 +5880,21 @@
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6921</v>
+        <v>7818</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>嘉雨思-創</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>187.9932954897044</v>
+        <v>191.0739285069669</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>63.7</v>
+        <v>63</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>47.42631558573308</v>
+        <v>35.60140952595299</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>26.81251412036929</v>
+        <v>33.29886568889377</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>1.350547815957848</v>
+        <v>0.5424617741357679</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.6906035743557759</v>
+        <v>-0.334856587748253</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>7760</v>
+        <v>6854</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>享溫馨</t>
+          <t>錼創科技-KY創</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>187.7116702053657</v>
+        <v>190.2200182423165</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>32.6</v>
+        <v>93.7</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>37.18368730295823</v>
+        <v>36.717587193692</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>14.34070556479804</v>
+        <v>38.9643703424982</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>2.86804293475812</v>
+        <v>0.2039096226856182</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.1941268720776278</v>
+        <v>1.47187137430882</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>7728</v>
+        <v>6921</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>嘉雨思-創</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>184.8778616436725</v>
+        <v>187.9932954897044</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>598</v>
+        <v>63.7</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>45.61913337951568</v>
+        <v>47.42631558573308</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>17.62611867654072</v>
+        <v>26.81251412036929</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.3889764886661511</v>
+        <v>1.350547815957848</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>5.629787691721226</v>
+        <v>0.6906035743557759</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>8032</v>
+        <v>7760</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>光菱</t>
+          <t>享溫馨</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>183.5331422848066</v>
+        <v>187.7116702053657</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>38.1</v>
+        <v>32.6</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,16 +6064,16 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>51.71591960974383</v>
+        <v>37.18368730295823</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>28.58192242599398</v>
+        <v>14.34070556479804</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>1.053375007901054</v>
+        <v>2.86804293475812</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.5561948324497608</v>
+        <v>-0.1941268720776278</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6962</v>
+        <v>7728</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>奕力-KY</t>
+          <t>光焱科技</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>182.0415059598681</v>
+        <v>184.8778616436725</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>33.8</v>
+        <v>598</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>52.80291368735963</v>
+        <v>45.61913337951568</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>24.84790768886231</v>
+        <v>17.62611867654072</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>1.466856451115353</v>
+        <v>0.3889764886661511</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.4296443780169021</v>
+        <v>5.629787691721226</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>8011</v>
+        <v>8032</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>台通</t>
+          <t>光菱</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>181.5514662356205</v>
+        <v>183.5331422848066</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>16.2</v>
+        <v>38.1</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,16 +6170,16 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>43.16223773266641</v>
+        <v>51.71591960974383</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>28.17824023911632</v>
+        <v>28.58192242599398</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.7859346886483324</v>
+        <v>1.053375007901054</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.0717313078149853</v>
+        <v>0.5561948324497608</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6909</v>
+        <v>6962</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>奕力-KY</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>178.8589365647425</v>
+        <v>182.0415059598681</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>40.8</v>
+        <v>33.8</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>39.70145188012542</v>
+        <v>52.80291368735963</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>29.36927703407951</v>
+        <v>24.84790768886231</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.5393359607652038</v>
+        <v>1.466856451115353</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.4119505155579985</v>
+        <v>0.4296443780169021</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6895</v>
+        <v>8011</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>宏碩系統</t>
+          <t>台通</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>175.4786785332464</v>
+        <v>181.5514662356205</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>118</v>
+        <v>16.2</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>37.97814902059178</v>
+        <v>43.16223773266641</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>25.52746731098111</v>
+        <v>28.17824023911632</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.3640786426271372</v>
+        <v>0.7859346886483324</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>1.159940731175791</v>
+        <v>0.0717313078149853</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6304,21 +6304,21 @@
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>7689</v>
+        <v>6909</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>大鵬科CLMX</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>174.8100905326966</v>
+        <v>178.8589365647425</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>173</v>
+        <v>40.8</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>29.96109749858409</v>
+        <v>39.70145188012542</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>32.01371027912507</v>
+        <v>29.36927703407951</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.7613588684964872</v>
+        <v>0.5393359607652038</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.1669219718625534</v>
+        <v>0.4119505155579985</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6357,21 +6357,21 @@
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>7823</v>
+        <v>6895</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>奧義賽博-KY創</t>
+          <t>宏碩系統</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>162.4137693956208</v>
+        <v>175.4786785332464</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>84.5</v>
+        <v>118</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>54.22799646309544</v>
+        <v>37.97814902059178</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>17.08652777136397</v>
+        <v>25.52746731098111</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.7272629349035942</v>
+        <v>0.3640786426271372</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.6244729802078971</v>
+        <v>1.159940731175791</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6908</v>
+        <v>7689</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>大鵬科CLMX</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>158.3204313107154</v>
+        <v>174.8100905326966</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>32.75</v>
+        <v>173</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>35.41562037522782</v>
+        <v>29.96109749858409</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>32.69032677099678</v>
+        <v>32.01371027912507</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>1.088792217227855</v>
+        <v>0.7613588684964872</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.0474432213775755</v>
+        <v>-0.1669219718625534</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6463,21 +6463,21 @@
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6885</v>
+        <v>7823</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>全福生技</t>
+          <t>奧義賽博-KY創</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>153.9165107969471</v>
+        <v>162.4137693956208</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>20.6</v>
+        <v>84.5</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>42.93095674182292</v>
+        <v>54.22799646309544</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>11.65423488581712</v>
+        <v>17.08652777136397</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.9764991879472044</v>
+        <v>0.7272629349035942</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0339135218299364</v>
+        <v>0.6244729802078971</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>7810</v>
+        <v>6908</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>捷創科技</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>147.3091756612734</v>
+        <v>158.3204313107154</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>196</v>
+        <v>32.75</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>50.99644362669503</v>
+        <v>35.41562037522782</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>15.0186828341978</v>
+        <v>32.69032677099678</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.4682805584904496</v>
+        <v>1.088792217227855</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>2.055460727840384</v>
+        <v>-0.0474432213775755</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>7765</v>
+        <v>6885</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>中華資安</t>
+          <t>全福生技</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>145.4235043508503</v>
+        <v>153.9165107969471</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>225.5</v>
+        <v>20.6</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>49.26095074954498</v>
+        <v>42.93095674182292</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>13.20100778128035</v>
+        <v>11.65423488581712</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.6405670336299201</v>
+        <v>0.9764991879472044</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.5713010948737607</v>
+        <v>0.0339135218299364</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6622,21 +6622,21 @@
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6983</v>
+        <v>7810</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>華洋精機</t>
+          <t>捷創科技</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>139.1063872733753</v>
+        <v>147.3091756612734</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>299</v>
+        <v>196</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>38.45100001245206</v>
+        <v>50.99644362669503</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>12.18775730209346</v>
+        <v>15.0186828341978</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.4791266892152341</v>
+        <v>0.4682805584904496</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.6193203675257415</v>
+        <v>2.055460727840384</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6923</v>
+        <v>7765</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>中華資安</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>131.2319260781561</v>
+        <v>145.4235043508503</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>74.90000000000001</v>
+        <v>225.5</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>45.45686190727599</v>
+        <v>49.26095074954498</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>10.24488373724783</v>
+        <v>13.20100778128035</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.5045807317500146</v>
+        <v>0.6405670336299201</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.0923619412484025</v>
+        <v>0.5713010948737607</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6728,21 +6728,21 @@
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6862</v>
+        <v>6983</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>華洋精機</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>117.5229661403532</v>
+        <v>139.1063872733753</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>148</v>
+        <v>299</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>46.68575204346558</v>
+        <v>38.45100001245206</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>20.92982672844532</v>
+        <v>12.18775730209346</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.7850170514899089</v>
+        <v>0.4791266892152341</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>3.273979148074696</v>
+        <v>0.6193203675257415</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6925</v>
+        <v>6923</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>意藍</t>
+          <t>中台</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>108.2954565029064</v>
+        <v>131.2319260781561</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>54.4</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>46.7552957503818</v>
+        <v>45.45686190727599</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.71965701541008</v>
+        <v>10.24488373724783</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.3576117077186561</v>
+        <v>0.5045807317500146</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.543195376086691</v>
+        <v>-0.0923619412484025</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>7703</v>
+        <v>6862</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>銳澤</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>83.00185572541767</v>
+        <v>117.5229661403532</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>179.5</v>
+        <v>148</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>48.48765582460498</v>
+        <v>46.68575204346558</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>19.38936541971981</v>
+        <v>20.92982672844532</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>1.259215539701856</v>
+        <v>0.7850170514899089</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>2.218340653792413</v>
+        <v>3.273979148074696</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>7753</v>
+        <v>6925</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>意藍</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>75.01819505146696</v>
+        <v>108.2954565029064</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>37.8</v>
+        <v>54.4</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>41.41569736151762</v>
+        <v>46.7552957503818</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>12.42134272569006</v>
+        <v>15.71965701541008</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.4394101270664969</v>
+        <v>0.3576117077186561</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0086600736524202</v>
+        <v>0.543195376086691</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,21 +6940,21 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6928</v>
+        <v>7703</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>攸泰科技</t>
+          <t>銳澤</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>72.80727720940872</v>
+        <v>83.00185572541767</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>48.5</v>
+        <v>179.5</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>46.42682475312564</v>
+        <v>48.48765582460498</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>15.28167911443106</v>
+        <v>19.38936541971981</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.2563829158291245</v>
+        <v>1.259215539701856</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.2797096613950488</v>
+        <v>2.218340653792413</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6971</v>
+        <v>7753</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>66.64156395903142</v>
+        <v>75.01819505146696</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>25.6</v>
+        <v>37.8</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>33.91237834119282</v>
+        <v>41.41569736151762</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>17.46445039138425</v>
+        <v>12.42134272569006</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.2963901860702075</v>
+        <v>0.4394101270664969</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.0597706896965913</v>
+        <v>-0.0086600736524202</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7046,21 +7046,21 @@
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>7736</v>
+        <v>6928</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>虎山</t>
+          <t>攸泰科技</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>64.14475539251939</v>
+        <v>72.80727720940872</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>70</v>
+        <v>48.5</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>44.05597008475656</v>
+        <v>46.42682475312564</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>17.34486392182579</v>
+        <v>15.28167911443106</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.097176458889838</v>
+        <v>0.2563829158291245</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.0363366732644843</v>
+        <v>-0.2797096613950488</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7099,52 +7099,158 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
+        <v>6971</v>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>惠民實業</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>66.64156395903142</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>33.91237834119282</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>17.46445039138425</v>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>0.2963901860702075</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N126" s="2" t="n">
+        <v>-0.0597706896965913</v>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>7736</v>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>虎山</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>64.14475539251939</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>44.05597008475656</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>17.34486392182579</v>
+      </c>
+      <c r="J127" s="2" t="n">
+        <v>0.097176458889838</v>
+      </c>
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
+        <v>0.0363366732644843</v>
+      </c>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="B126" s="2" t="inlineStr">
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>君曜</t>
         </is>
       </c>
-      <c r="C126" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D126" s="2" t="n">
+      <c r="C128" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D128" s="2" t="n">
         <v>9.482355299335548</v>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E128" s="2" t="n">
         <v>39.75</v>
       </c>
-      <c r="F126" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="G126" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H126" s="2" t="n">
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H128" s="2" t="n">
         <v>52.28709349733273</v>
       </c>
-      <c r="I126" s="2" t="n">
+      <c r="I128" s="2" t="n">
         <v>12.34638549130708</v>
       </c>
-      <c r="J126" s="2" t="n">
+      <c r="J128" s="2" t="n">
         <v>0.1990832459309326</v>
       </c>
-      <c r="K126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M126" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N126" s="2" t="n">
+      <c r="K128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N128" s="2" t="n">
         <v>1.10788863669533</v>
       </c>
-      <c r="O126" s="2" t="inlineStr">
+      <c r="O128" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, mfi_strong</t>
         </is>

</xml_diff>

<commit_message>
scan: seg7 2026-08-11 18:02 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-08-11.xlsx
+++ b/output/full_scan/batch_seq8_2026-08-11.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O128"/>
+  <dimension ref="A1:O129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5350,21 +5350,21 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6934</v>
+        <v>7828</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>心誠鎂</t>
+          <t>創新服務</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>222.6470469207084</v>
+        <v>225.1037090936148</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>72.5</v>
+        <v>1605</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,16 +5375,16 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>44.4856215316977</v>
+        <v>46.06294024641603</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>17.36267837071677</v>
+        <v>15.82499428187163</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>1.198601973684211</v>
+        <v>0.4878220499115206</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.7611766531987858</v>
+        <v>12.43847583872932</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>8024</v>
+        <v>6934</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>佑華</t>
+          <t>心誠鎂</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>220.1334953149262</v>
+        <v>222.6470469207084</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>13.8</v>
+        <v>72.5</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>41.71054769576779</v>
+        <v>44.4856215316977</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>17.34720052770448</v>
+        <v>17.36267837071677</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.753759353792649</v>
+        <v>1.198601973684211</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.1463191595500006</v>
+        <v>-0.7611766531987858</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>7842</v>
+        <v>8024</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>佑華</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>212.7984579954426</v>
+        <v>220.1334953149262</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>94</v>
+        <v>13.8</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>54.31749663823657</v>
+        <v>41.71054769576779</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>10.66722445620016</v>
+        <v>17.34720052770448</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>3.21661227373806</v>
+        <v>0.753759353792649</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>1.907900389183593</v>
+        <v>-0.1463191595500006</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6887</v>
+        <v>7842</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>寶綠特-KY</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>211.68617814312</v>
+        <v>212.7984579954426</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>36.45</v>
+        <v>94</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>49.31695248432469</v>
+        <v>54.31749663823657</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>17.04578355064413</v>
+        <v>10.66722445620016</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.1825626148277355</v>
+        <v>3.21661227373806</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.1819288498890896</v>
+        <v>1.907900389183593</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6894</v>
+        <v>6887</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>衛司特</t>
+          <t>寶綠特-KY</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>208.873830439202</v>
+        <v>211.68617814312</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>345</v>
+        <v>36.45</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>52.3219923856823</v>
+        <v>49.31695248432469</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>15.45647148628926</v>
+        <v>17.04578355064413</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.8203025307091175</v>
+        <v>0.1825626148277355</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>4.056701308693365</v>
+        <v>-0.1819288498890896</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6916</v>
+        <v>6894</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>衛司特</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>204.5744204188318</v>
+        <v>208.873830439202</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>18.7</v>
+        <v>345</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>47.58853670104529</v>
+        <v>52.3219923856823</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>13.81213421387869</v>
+        <v>15.45647148628926</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.200521903827872</v>
+        <v>0.8203025307091175</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.0527311534019029</v>
+        <v>4.056701308693365</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5668,21 +5668,21 @@
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6953</v>
+        <v>6916</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>204.1981402739606</v>
+        <v>204.5744204188318</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>220.5</v>
+        <v>18.7</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>51.07536084264394</v>
+        <v>47.58853670104529</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>9.407512687987516</v>
+        <v>13.81213421387869</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.1880072290599755</v>
+        <v>0.200521903827872</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>2.04210416579964</v>
+        <v>0.0527311534019029</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6988</v>
+        <v>6953</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>威力暘-創</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>203.5494061530428</v>
+        <v>204.1981402739606</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>12.7</v>
+        <v>220.5</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>50.98520902686534</v>
+        <v>51.07536084264394</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>10.68239455268137</v>
+        <v>9.407512687987516</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.9285713101312104</v>
+        <v>0.1880072290599755</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.2437915569015741</v>
+        <v>2.04210416579964</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, kd_golden_cross, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6899</v>
+        <v>6988</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>威力暘-創</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>203.317649325788</v>
+        <v>203.5494061530428</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>51</v>
+        <v>12.7</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>40.48779896859401</v>
+        <v>50.98520902686534</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>22.59476417999487</v>
+        <v>10.68239455268137</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.5579291095827936</v>
+        <v>0.9285713101312104</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.3811609168553613</v>
+        <v>0.2437915569015741</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>7791</v>
+        <v>6899</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>195.5050053759604</v>
+        <v>203.317649325788</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>59.5</v>
+        <v>51</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>31.9038991525452</v>
+        <v>40.48779896859401</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>25.76078683036973</v>
+        <v>22.59476417999487</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.424318686171579</v>
+        <v>0.5579291095827936</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.08340806992414471</v>
+        <v>0.3811609168553613</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5880,21 +5880,21 @@
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>7818</v>
+        <v>7791</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>191.0739285069669</v>
+        <v>195.5050053759604</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>63</v>
+        <v>59.5</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>35.60140952595299</v>
+        <v>31.9038991525452</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>33.29886568889377</v>
+        <v>25.76078683036973</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.5424617741357679</v>
+        <v>0.424318686171579</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.334856587748253</v>
+        <v>-0.08340806992414471</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5933,21 +5933,21 @@
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6854</v>
+        <v>7818</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>190.2200182423165</v>
+        <v>191.0739285069669</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>93.7</v>
+        <v>63</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>36.717587193692</v>
+        <v>35.60140952595299</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>38.9643703424982</v>
+        <v>33.29886568889377</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.2039096226856182</v>
+        <v>0.5424617741357679</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>1.47187137430882</v>
+        <v>-0.334856587748253</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5986,21 +5986,21 @@
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6921</v>
+        <v>6854</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>嘉雨思-創</t>
+          <t>錼創科技-KY創</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>187.9932954897044</v>
+        <v>190.2200182423165</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>63.7</v>
+        <v>93.7</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>47.42631558573308</v>
+        <v>36.717587193692</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>26.81251412036929</v>
+        <v>38.9643703424982</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>1.350547815957848</v>
+        <v>0.2039096226856182</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.6906035743557759</v>
+        <v>1.47187137430882</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>7760</v>
+        <v>6921</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>享溫馨</t>
+          <t>嘉雨思-創</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>187.7116702053657</v>
+        <v>187.9932954897044</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>32.6</v>
+        <v>63.7</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>37.18368730295823</v>
+        <v>47.42631558573308</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>14.34070556479804</v>
+        <v>26.81251412036929</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>2.86804293475812</v>
+        <v>1.350547815957848</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.1941268720776278</v>
+        <v>0.6906035743557759</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>7728</v>
+        <v>7760</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>享溫馨</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>184.8778616436725</v>
+        <v>187.7116702053657</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>598</v>
+        <v>32.6</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>45.61913337951568</v>
+        <v>37.18368730295823</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>17.62611867654072</v>
+        <v>14.34070556479804</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.3889764886661511</v>
+        <v>2.86804293475812</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>5.629787691721226</v>
+        <v>-0.1941268720776278</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>8032</v>
+        <v>7728</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>光菱</t>
+          <t>光焱科技</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>183.5331422848066</v>
+        <v>184.8778616436725</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>38.1</v>
+        <v>598</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,16 +6170,16 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>51.71591960974383</v>
+        <v>45.61913337951568</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>28.58192242599398</v>
+        <v>17.62611867654072</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>1.053375007901054</v>
+        <v>0.3889764886661511</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.5561948324497608</v>
+        <v>5.629787691721226</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6962</v>
+        <v>8032</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>奕力-KY</t>
+          <t>光菱</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>182.0415059598681</v>
+        <v>183.5331422848066</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>33.8</v>
+        <v>38.1</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,16 +6223,16 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>52.80291368735963</v>
+        <v>51.71591960974383</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>24.84790768886231</v>
+        <v>28.58192242599398</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>1.466856451115353</v>
+        <v>1.053375007901054</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.4296443780169021</v>
+        <v>0.5561948324497608</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>8011</v>
+        <v>6962</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>台通</t>
+          <t>奕力-KY</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>181.5514662356205</v>
+        <v>182.0415059598681</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>16.2</v>
+        <v>33.8</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>43.16223773266641</v>
+        <v>52.80291368735963</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>28.17824023911632</v>
+        <v>24.84790768886231</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.7859346886483324</v>
+        <v>1.466856451115353</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.0717313078149853</v>
+        <v>0.4296443780169021</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6909</v>
+        <v>8011</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>台通</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>178.8589365647425</v>
+        <v>181.5514662356205</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>40.8</v>
+        <v>16.2</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>39.70145188012542</v>
+        <v>43.16223773266641</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>29.36927703407951</v>
+        <v>28.17824023911632</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.5393359607652038</v>
+        <v>0.7859346886483324</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.4119505155579985</v>
+        <v>0.0717313078149853</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6357,21 +6357,21 @@
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6895</v>
+        <v>6909</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>宏碩系統</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>175.4786785332464</v>
+        <v>178.8589365647425</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>118</v>
+        <v>40.8</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>37.97814902059178</v>
+        <v>39.70145188012542</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>25.52746731098111</v>
+        <v>29.36927703407951</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.3640786426271372</v>
+        <v>0.5393359607652038</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>1.159940731175791</v>
+        <v>0.4119505155579985</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6410,21 +6410,21 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>7689</v>
+        <v>6895</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>大鵬科CLMX</t>
+          <t>宏碩系統</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>174.8100905326966</v>
+        <v>175.4786785332464</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>173</v>
+        <v>118</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>29.96109749858409</v>
+        <v>37.97814902059178</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>32.01371027912507</v>
+        <v>25.52746731098111</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.7613588684964872</v>
+        <v>0.3640786426271372</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.1669219718625534</v>
+        <v>1.159940731175791</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6463,21 +6463,21 @@
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>7823</v>
+        <v>7689</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>奧義賽博-KY創</t>
+          <t>大鵬科CLMX</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>162.4137693956208</v>
+        <v>174.8100905326966</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>84.5</v>
+        <v>173</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>54.22799646309544</v>
+        <v>29.96109749858409</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>17.08652777136397</v>
+        <v>32.01371027912507</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.7272629349035942</v>
+        <v>0.7613588684964872</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.6244729802078971</v>
+        <v>-0.1669219718625534</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6908</v>
+        <v>7823</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>奧義賽博-KY創</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>158.3204313107154</v>
+        <v>162.4137693956208</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>32.75</v>
+        <v>84.5</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>35.41562037522782</v>
+        <v>54.22799646309544</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>32.69032677099678</v>
+        <v>17.08652777136397</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>1.088792217227855</v>
+        <v>0.7272629349035942</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0474432213775755</v>
+        <v>0.6244729802078971</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6885</v>
+        <v>6908</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>全福生技</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>153.9165107969471</v>
+        <v>158.3204313107154</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>20.6</v>
+        <v>32.75</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>42.93095674182292</v>
+        <v>35.41562037522782</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>11.65423488581712</v>
+        <v>32.69032677099678</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.9764991879472044</v>
+        <v>1.088792217227855</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0339135218299364</v>
+        <v>-0.0474432213775755</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>7810</v>
+        <v>6885</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>捷創科技</t>
+          <t>全福生技</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>147.3091756612734</v>
+        <v>153.9165107969471</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>196</v>
+        <v>20.6</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>50.99644362669503</v>
+        <v>42.93095674182292</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>15.0186828341978</v>
+        <v>11.65423488581712</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.4682805584904496</v>
+        <v>0.9764991879472044</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>2.055460727840384</v>
+        <v>0.0339135218299364</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6675,21 +6675,21 @@
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>7765</v>
+        <v>7810</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>中華資安</t>
+          <t>捷創科技</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>145.4235043508503</v>
+        <v>147.3091756612734</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>225.5</v>
+        <v>196</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>49.26095074954498</v>
+        <v>50.99644362669503</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>13.20100778128035</v>
+        <v>15.0186828341978</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.6405670336299201</v>
+        <v>0.4682805584904496</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.5713010948737607</v>
+        <v>2.055460727840384</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6728,21 +6728,21 @@
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6983</v>
+        <v>7765</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>華洋精機</t>
+          <t>中華資安</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>139.1063872733753</v>
+        <v>145.4235043508503</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>299</v>
+        <v>225.5</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>38.45100001245206</v>
+        <v>49.26095074954498</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>12.18775730209346</v>
+        <v>13.20100778128035</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.4791266892152341</v>
+        <v>0.6405670336299201</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.6193203675257415</v>
+        <v>0.5713010948737607</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6923</v>
+        <v>6983</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>華洋精機</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>131.2319260781561</v>
+        <v>139.1063872733753</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>74.90000000000001</v>
+        <v>299</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>45.45686190727599</v>
+        <v>38.45100001245206</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>10.24488373724783</v>
+        <v>12.18775730209346</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.5045807317500146</v>
+        <v>0.4791266892152341</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,31 +6824,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.0923619412484025</v>
+        <v>0.6193203675257415</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6862</v>
+        <v>6923</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>中台</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>117.5229661403532</v>
+        <v>131.2319260781561</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>148</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,13 +6859,13 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>46.68575204346558</v>
+        <v>45.45686190727599</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>20.92982672844532</v>
+        <v>10.24488373724783</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.7850170514899089</v>
+        <v>0.5045807317500146</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>3.273979148074696</v>
+        <v>-0.0923619412484025</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6925</v>
+        <v>6862</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>意藍</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>108.2954565029064</v>
+        <v>117.5229661403532</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>54.4</v>
+        <v>148</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>46.7552957503818</v>
+        <v>46.68575204346558</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>15.71965701541008</v>
+        <v>20.92982672844532</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.3576117077186561</v>
+        <v>0.7850170514899089</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,31 +6930,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.543195376086691</v>
+        <v>3.273979148074696</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>7703</v>
+        <v>6925</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>銳澤</t>
+          <t>意藍</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>83.00185572541767</v>
+        <v>108.2954565029064</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>179.5</v>
+        <v>54.4</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>48.48765582460498</v>
+        <v>46.7552957503818</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>19.38936541971981</v>
+        <v>15.71965701541008</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>1.259215539701856</v>
+        <v>0.3576117077186561</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>2.218340653792413</v>
+        <v>0.543195376086691</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>7753</v>
+        <v>7703</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>銳澤</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>75.01819505146696</v>
+        <v>83.00185572541767</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>37.8</v>
+        <v>179.5</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,16 +7018,16 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>41.41569736151762</v>
+        <v>48.48765582460498</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>12.42134272569006</v>
+        <v>19.38936541971981</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.4394101270664969</v>
+        <v>1.259215539701856</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.0086600736524202</v>
+        <v>2.218340653792413</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6928</v>
+        <v>7753</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>攸泰科技</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>72.80727720940872</v>
+        <v>75.01819505146696</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>48.5</v>
+        <v>37.8</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>46.42682475312564</v>
+        <v>41.41569736151762</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>15.28167911443106</v>
+        <v>12.42134272569006</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.2563829158291245</v>
+        <v>0.4394101270664969</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.2797096613950488</v>
+        <v>-0.0086600736524202</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7099,21 +7099,21 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>6971</v>
+        <v>6928</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>攸泰科技</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>66.64156395903142</v>
+        <v>72.80727720940872</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>25.6</v>
+        <v>48.5</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,13 +7124,13 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>33.91237834119282</v>
+        <v>46.42682475312564</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>17.46445039138425</v>
+        <v>15.28167911443106</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.2963901860702075</v>
+        <v>0.2563829158291245</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>0</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.0597706896965913</v>
+        <v>-0.2797096613950488</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7152,21 +7152,21 @@
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>7736</v>
+        <v>6971</v>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>虎山</t>
+          <t>惠民實業</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>64.14475539251939</v>
+        <v>66.64156395903142</v>
       </c>
       <c r="E127" s="2" t="n">
-        <v>70</v>
+        <v>25.6</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -7177,13 +7177,13 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>44.05597008475656</v>
+        <v>33.91237834119282</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>17.34486392182579</v>
+        <v>17.46445039138425</v>
       </c>
       <c r="J127" s="2" t="n">
-        <v>0.097176458889838</v>
+        <v>0.2963901860702075</v>
       </c>
       <c r="K127" s="2" t="n">
         <v>0</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>0.0363366732644843</v>
+        <v>-0.0597706896965913</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7205,52 +7205,105 @@
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
+        <v>7736</v>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>虎山</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D128" s="2" t="n">
+        <v>64.14475539251939</v>
+      </c>
+      <c r="E128" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H128" s="2" t="n">
+        <v>44.05597008475656</v>
+      </c>
+      <c r="I128" s="2" t="n">
+        <v>17.34486392182579</v>
+      </c>
+      <c r="J128" s="2" t="n">
+        <v>0.097176458889838</v>
+      </c>
+      <c r="K128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N128" s="2" t="n">
+        <v>0.0363366732644843</v>
+      </c>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="B128" s="2" t="inlineStr">
+      <c r="B129" s="2" t="inlineStr">
         <is>
           <t>君曜</t>
         </is>
       </c>
-      <c r="C128" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D128" s="2" t="n">
+      <c r="C129" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D129" s="2" t="n">
         <v>9.482355299335548</v>
       </c>
-      <c r="E128" s="2" t="n">
+      <c r="E129" s="2" t="n">
         <v>39.75</v>
       </c>
-      <c r="F128" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="G128" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H128" s="2" t="n">
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H129" s="2" t="n">
         <v>52.28709349733273</v>
       </c>
-      <c r="I128" s="2" t="n">
+      <c r="I129" s="2" t="n">
         <v>12.34638549130708</v>
       </c>
-      <c r="J128" s="2" t="n">
+      <c r="J129" s="2" t="n">
         <v>0.1990832459309326</v>
       </c>
-      <c r="K128" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L128" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M128" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N128" s="2" t="n">
+      <c r="K129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M129" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N129" s="2" t="n">
         <v>1.10788863669533</v>
       </c>
-      <c r="O128" s="2" t="inlineStr">
+      <c r="O129" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, mfi_strong</t>
         </is>

</xml_diff>